<commit_message>
Conveyor more parameters added and vibrating feeder updates
</commit_message>
<xml_diff>
--- a/backend/excel/Bearing Life Calculator.xlsx
+++ b/backend/excel/Bearing Life Calculator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showObjects="none"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BIT\Desktop\SAIL\Bearing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BIT\Desktop\SAIL\mechanical-calculator\backend\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668A978B-FB44-47F5-AE52-92EFF6EE1612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7C1D87-AE93-4E9B-9BDD-27F31CCB477F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bearing Life Calculator" sheetId="1" r:id="rId1"/>
@@ -1625,7 +1625,8 @@
         <v>25</v>
       </c>
       <c r="B10">
-        <v>10000</v>
+        <f>'Bearing Life Calculator'!C12</f>
+        <v>30000</v>
       </c>
       <c r="C10" t="s">
         <v>17</v>
@@ -1635,7 +1636,7 @@
       </c>
       <c r="F10">
         <f>B10/B12</f>
-        <v>32.520325203252035</v>
+        <v>97.560975609756099</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -1654,7 +1655,7 @@
       </c>
       <c r="F11">
         <f>B10/B11</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>